<commit_message>
fix analyses, translate to English, add RQ3 tables
</commit_message>
<xml_diff>
--- a/results/RQ1/comparison_categories.xlsx
+++ b/results/RQ1/comparison_categories.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,382 +417,382 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Categoria</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Facilidade</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Efetividade</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Frequencia</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Essencialidade</t>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ease of use</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Effectiveness</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Frequency of use</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Essentiality</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Revisão de Código</t>
+          <t>Code Review</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7118189073496337</v>
+        <v>0.7111111111111111</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8273348519362188</v>
+        <v>0.8453333333333334</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7790460730814394</v>
+        <v>0.78</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8899463639765498</v>
+        <v>0.8891566265060241</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Modelagem de Ameaças</t>
+          <t>Threat Modeling</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.6449399922570654</v>
+        <v>0.6476190476190476</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8170323928944617</v>
+        <v>0.8276923076923077</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6844758918735701</v>
+        <v>0.6754385964912281</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8530497692403641</v>
+        <v>0.8457831325301205</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Identificação de Casos de Abuso/Mau Uso</t>
+          <t>Identifying Abuse/Misuse Cases</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.6179581795817959</v>
+        <v>0.6</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7491962805449434</v>
+        <v>0.7681159420289855</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7407100644699141</v>
+        <v>0.7129629629629629</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8081077709866533</v>
+        <v>0.8096385542168675</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Análise de Riscos Arquiteturais</t>
+          <t>Architectural Risk Analysis</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.6131407533276692</v>
+        <v>0.6</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8179501385041552</v>
+        <v>0.8366197183098592</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6539196940726577</v>
+        <v>0.6388888888888888</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8540476487464138</v>
+        <v>0.8506024096385543</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Testes de Penetração</t>
+          <t>Penetration Testing</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6423696615774291</v>
+        <v>0.6352941176470588</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8794044321329638</v>
+        <v>0.8753623188405797</v>
       </c>
       <c r="E6" t="n">
-        <v>0.5911096156721998</v>
+        <v>0.5766129032258065</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8876886615941123</v>
+        <v>0.8722891566265061</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gerenciamento de Riscos</t>
+          <t>Risk Management</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6231487708286633</v>
+        <v>0.6246153846153846</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8406507500528207</v>
+        <v>0.8521739130434782</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6947547353084023</v>
+        <v>0.6833333333333333</v>
       </c>
       <c r="F7" t="n">
-        <v>0.8778346014718721</v>
+        <v>0.8746987951807229</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gerenciamento de Vulnerabilidades</t>
+          <t>Vulnerability Management</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.7041602465331277</v>
+        <v>0.7</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8538734516237025</v>
+        <v>0.8602739726027397</v>
       </c>
       <c r="E8" t="n">
-        <v>0.81404360107192</v>
+        <v>0.7934782608695652</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8993887988025445</v>
+        <v>0.8987951807228916</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Testes de Segurança Manuais/Automatizados</t>
+          <t>Manual/Automated Security Testing</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6825869262865091</v>
+        <v>0.68</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8219806926348477</v>
+        <v>0.8328767123287671</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7588428845626544</v>
+        <v>0.75</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8654359486092055</v>
+        <v>0.8602409638554217</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Execução de Testes Fuzz</t>
+          <t>Performing Fuzz Testing</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.6265875785066295</v>
+        <v>0.6327272727272727</v>
       </c>
       <c r="D10" t="n">
-        <v>0.6525466139317138</v>
+        <v>0.6711864406779661</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6963842333954068</v>
+        <v>0.6976744186046512</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6701384557814644</v>
+        <v>0.6771084337349398</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Engenharia de Requisitos de Segurança</t>
+          <t>Security Requirements Engineering</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6331731136034179</v>
+        <v>0.638095238095238</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8149410595085925</v>
+        <v>0.8376811594202899</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6706680126404494</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8272795309966321</v>
+        <v>0.8240963855421687</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Codificação Segura</t>
+          <t>Secure Coding</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.6592795186371806</v>
+        <v>0.6615384615384615</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8522785768357305</v>
+        <v>0.8757575757575757</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8143000250438266</v>
+        <v>0.819672131147541</v>
       </c>
       <c r="F12" t="n">
-        <v>0.899239116876637</v>
+        <v>0.8939759036144578</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Resposta Emergencial ao Código</t>
+          <t>Emergency Codebase Response</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.6021140878439949</v>
+        <v>0.6072727272727273</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7238119746097099</v>
+        <v>0.7413793103448276</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7369499063670414</v>
+        <v>0.7261904761904762</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7619059498565548</v>
+        <v>0.7686746987951807</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Configurações e Gerenciamento de Segurança</t>
+          <t>Security Configurations &amp; Management</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.6623842246788171</v>
+        <v>0.6636363636363637</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8098529521534674</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="E14" t="n">
-        <v>0.7456107031315946</v>
+        <v>0.7330508474576272</v>
       </c>
       <c r="F14" t="n">
-        <v>0.8560808282399899</v>
+        <v>0.8554216867469879</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Monitoramento de Eventos de Segurança</t>
+          <t>Monitoring for Security Events</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.6423446105428796</v>
+        <v>0.65</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8709259947936034</v>
+        <v>0.8835820895522388</v>
       </c>
       <c r="E15" t="n">
-        <v>0.7913708127975942</v>
+        <v>0.7833333333333333</v>
       </c>
       <c r="F15" t="n">
-        <v>0.8744418111513034</v>
+        <v>0.8819277108433735</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Auditorias de Segurança Externas</t>
+          <t>Undergoing External Security Audits</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.6300500287049947</v>
+        <v>0.6275862068965518</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7123809523809524</v>
+        <v>0.7278688524590164</v>
       </c>
       <c r="E16" t="n">
-        <v>0.5053494352098448</v>
+        <v>0.4803921568627451</v>
       </c>
       <c r="F16" t="n">
-        <v>0.747623799426219</v>
+        <v>0.7518072289156627</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Segurança da Cadeia de Suprimentos de Software</t>
+          <t>Software Supply Chain Security</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.6114271661611609</v>
+        <v>0.6137931034482759</v>
       </c>
       <c r="D17" t="n">
-        <v>0.7802486622599936</v>
+        <v>0.780327868852459</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6955769413103252</v>
+        <v>0.6836734693877551</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8352376200573778</v>
+        <v>0.8216867469879519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>